<commit_message>
Add execution logs, outputs and main runner
Add generated execution logs and update pipeline outputs from a full run: new LOGS/*.txt, updated OUTPUT_3.1_TRATAMENTO, OUTPUT_3.2.b_CBR_TESTS, OUTPUT_3.3.* and OUTPUT_3.4 directories (plots, Excel sheets, .mat models and imputed datasets). Also add tp_main.m and update tp_main_run_all.m and tp_3_3_a_RN_implementacao.m to include/drive the full experiment run. These changes are artifacts of running the data treatment, CBR retrieval, and neural-network testing pipeline and capture resulting reports and figures.
</commit_message>
<xml_diff>
--- a/Trabalho M2/OUTPUT_3.3.a_RN_IMPL/Common/Resultados_Estudo_Parametrico.xlsx
+++ b/Trabalho M2/OUTPUT_3.3.a_RN_IMPL/Common/Resultados_Estudo_Parametrico.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="292" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="1096" uniqueCount="79">
   <si>
     <t>rank</t>
   </si>
@@ -148,6 +148,108 @@
   </si>
   <si>
     <t>avg_tr_time</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainscg_softmax_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainlm_logsig_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-5-5_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainlm_softmax_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-10_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-10_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-10_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-5-5_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainscg_softmax_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainlm_logsig_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-10_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-10_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainlm_softmax_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-5-5_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainlm_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-5-5_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-10_trainscg_softmax_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainscg_logsig_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-10_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-14_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-10_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainscg_logsig_MF6_Div-0.7-0.15-0.15</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-5-5_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-14_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_MICE_NORM_Topo-5-5_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-5-5_trainlm_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>RN_Median_NORM_Topo-5-5_trainscg_logsig_MF6_Div-0.6-0.2-0.2</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>[0.6 0.2 0.2]</t>
   </si>
 </sst>
 </file>
@@ -193,7 +295,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R17"/>
+  <dimension ref="A1:R49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="4.6328125" customWidth="true"/>
@@ -213,7 +315,7 @@
     <col min="15" max="15" width="11.453125" customWidth="true"/>
     <col min="16" max="16" width="15.453125" customWidth="true"/>
     <col min="17" max="17" width="14.36328125" customWidth="true"/>
-    <col min="18" max="18" width="12.453125" customWidth="true"/>
+    <col min="18" max="18" width="10.81640625" customWidth="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -277,7 +379,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="0" t="s">
-        <v>2</v>
+        <v>46</v>
       </c>
       <c r="C2" s="0" t="s">
         <v>19</v>
@@ -286,7 +388,7 @@
         <v>22</v>
       </c>
       <c r="E2" s="0" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F2" s="0" t="s">
         <v>27</v>
@@ -298,34 +400,34 @@
         <v>32</v>
       </c>
       <c r="I2" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J2" s="0">
         <v>6</v>
       </c>
       <c r="K2" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L2" s="0">
-        <v>16.669396181788564</v>
+        <v>16.671971391100136</v>
       </c>
       <c r="M2" s="0">
-        <v>16.67233487171676</v>
+        <v>16.675301017484905</v>
       </c>
       <c r="N2" s="0">
-        <v>99.993333333333339</v>
+        <v>99.977999999999995</v>
       </c>
       <c r="O2" s="0">
-        <v>100</v>
+        <v>99.989999999999995</v>
       </c>
       <c r="P2" s="0">
-        <v>20</v>
+        <v>22.699999999999999</v>
       </c>
       <c r="Q2" s="0">
-        <v>16</v>
+        <v>18.5</v>
       </c>
       <c r="R2" s="0">
-        <v>0.46633333333333366</v>
+        <v>0.73570000000000069</v>
       </c>
     </row>
     <row r="3">
@@ -333,7 +435,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>19</v>
@@ -342,10 +444,10 @@
         <v>22</v>
       </c>
       <c r="E3" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F3" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G3" s="0" t="s">
         <v>30</v>
@@ -360,28 +462,28 @@
         <v>6</v>
       </c>
       <c r="K3" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L3" s="0">
-        <v>16.670574079582504</v>
+        <v>16.680103682126081</v>
       </c>
       <c r="M3" s="0">
-        <v>16.678924332295239</v>
+        <v>16.684390614019716</v>
       </c>
       <c r="N3" s="0">
-        <v>99.986666666666679</v>
+        <v>99.974000000000004</v>
       </c>
       <c r="O3" s="0">
-        <v>99.955555555555563</v>
+        <v>99.960000000000008</v>
       </c>
       <c r="P3" s="0">
-        <v>80</v>
+        <v>32.299999999999997</v>
       </c>
       <c r="Q3" s="0">
-        <v>75.333333333333329</v>
+        <v>28.5</v>
       </c>
       <c r="R3" s="0">
-        <v>2.0589999999999975</v>
+        <v>0.30399999999999994</v>
       </c>
     </row>
     <row r="4">
@@ -389,7 +491,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="C4" s="0" t="s">
         <v>19</v>
@@ -401,7 +503,7 @@
         <v>24</v>
       </c>
       <c r="F4" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G4" s="0" t="s">
         <v>30</v>
@@ -410,34 +512,34 @@
         <v>33</v>
       </c>
       <c r="I4" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J4" s="0">
         <v>6</v>
       </c>
       <c r="K4" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L4" s="0">
-        <v>16.672893379763796</v>
+        <v>16.680005763376833</v>
       </c>
       <c r="M4" s="0">
-        <v>16.688859998636449</v>
+        <v>16.688197871479059</v>
       </c>
       <c r="N4" s="0">
-        <v>99.980000000000004</v>
+        <v>99.970000000000013</v>
       </c>
       <c r="O4" s="0">
-        <v>99.911111111111112</v>
+        <v>99.949999999999989</v>
       </c>
       <c r="P4" s="0">
-        <v>23</v>
+        <v>30.100000000000001</v>
       </c>
       <c r="Q4" s="0">
-        <v>17</v>
+        <v>26.800000000000001</v>
       </c>
       <c r="R4" s="0">
-        <v>0.53433333333333388</v>
+        <v>0.27639999999999992</v>
       </c>
     </row>
     <row r="5">
@@ -445,7 +547,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>19</v>
@@ -457,13 +559,13 @@
         <v>24</v>
       </c>
       <c r="F5" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G5" s="0" t="s">
         <v>30</v>
       </c>
       <c r="H5" s="0" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I5" s="0" t="s">
         <v>35</v>
@@ -472,28 +574,28 @@
         <v>6</v>
       </c>
       <c r="K5" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L5" s="0">
-        <v>16.675649680248103</v>
+        <v>16.670444338654345</v>
       </c>
       <c r="M5" s="0">
-        <v>16.701777716024285</v>
+        <v>16.676697681172556</v>
       </c>
       <c r="N5" s="0">
-        <v>99.980000000000004</v>
+        <v>99.986000000000018</v>
       </c>
       <c r="O5" s="0">
-        <v>99.911111111111112</v>
+        <v>99.946666666666673</v>
       </c>
       <c r="P5" s="0">
-        <v>33.666666666666664</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="Q5" s="0">
-        <v>31.666666666666668</v>
+        <v>16.5</v>
       </c>
       <c r="R5" s="0">
-        <v>0.30399999999999733</v>
+        <v>0.45020000000000027</v>
       </c>
     </row>
     <row r="6">
@@ -501,7 +603,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>19</v>
@@ -510,7 +612,7 @@
         <v>22</v>
       </c>
       <c r="E6" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" s="0" t="s">
         <v>27</v>
@@ -519,7 +621,7 @@
         <v>30</v>
       </c>
       <c r="H6" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I6" s="0" t="s">
         <v>35</v>
@@ -528,28 +630,28 @@
         <v>6</v>
       </c>
       <c r="K6" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L6" s="0">
-        <v>16.674198687528989</v>
+        <v>16.689561188192052</v>
       </c>
       <c r="M6" s="0">
-        <v>16.704911156032423</v>
+        <v>16.70507316504634</v>
       </c>
       <c r="N6" s="0">
-        <v>99.973333333333343</v>
+        <v>99.944000000000003</v>
       </c>
       <c r="O6" s="0">
-        <v>99.866666666666674</v>
+        <v>99.906666666666666</v>
       </c>
       <c r="P6" s="0">
-        <v>25.666666666666668</v>
+        <v>15.4</v>
       </c>
       <c r="Q6" s="0">
-        <v>23.666666666666668</v>
+        <v>9.4000000000000004</v>
       </c>
       <c r="R6" s="0">
-        <v>0.64266666666666816</v>
+        <v>0.37900000000000062</v>
       </c>
     </row>
     <row r="7">
@@ -557,7 +659,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>14</v>
+        <v>52</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>19</v>
@@ -566,10 +668,10 @@
         <v>22</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F7" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G7" s="0" t="s">
         <v>30</v>
@@ -578,34 +680,34 @@
         <v>33</v>
       </c>
       <c r="I7" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J7" s="0">
         <v>6</v>
       </c>
       <c r="K7" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L7" s="0">
-        <v>16.701333714873631</v>
+        <v>16.679568561466468</v>
       </c>
       <c r="M7" s="0">
-        <v>16.718421096041748</v>
+        <v>16.701808280046052</v>
       </c>
       <c r="N7" s="0">
-        <v>99.933333333333337</v>
+        <v>99.968000000000004</v>
       </c>
       <c r="O7" s="0">
-        <v>99.866666666666674</v>
+        <v>99.899999999999991</v>
       </c>
       <c r="P7" s="0">
-        <v>33.333333333333336</v>
+        <v>37</v>
       </c>
       <c r="Q7" s="0">
-        <v>28.333333333333332</v>
+        <v>31</v>
       </c>
       <c r="R7" s="0">
-        <v>0.46733333333333338</v>
+        <v>0.92820000000000069</v>
       </c>
     </row>
     <row r="8">
@@ -613,16 +715,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="C8" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D8" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="F8" s="0" t="s">
         <v>27</v>
@@ -634,34 +736,34 @@
         <v>33</v>
       </c>
       <c r="I8" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J8" s="0">
         <v>6</v>
       </c>
       <c r="K8" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L8" s="0">
-        <v>16.745137798403178</v>
+        <v>16.678524640021489</v>
       </c>
       <c r="M8" s="0">
-        <v>16.778712698593949</v>
+        <v>16.704462788220901</v>
       </c>
       <c r="N8" s="0">
-        <v>99.779999999999987</v>
+        <v>99.968000000000004</v>
       </c>
       <c r="O8" s="0">
-        <v>99.644444444444446</v>
+        <v>99.890000000000001</v>
       </c>
       <c r="P8" s="0">
-        <v>27.333333333333332</v>
+        <v>51.399999999999999</v>
       </c>
       <c r="Q8" s="0">
-        <v>21.333333333333332</v>
+        <v>46</v>
       </c>
       <c r="R8" s="0">
-        <v>0.68199999999999983</v>
+        <v>1.6949000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -669,10 +771,10 @@
         <v>8</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>7</v>
+        <v>55</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D9" s="0" t="s">
         <v>22</v>
@@ -681,7 +783,7 @@
         <v>25</v>
       </c>
       <c r="F9" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G9" s="0" t="s">
         <v>30</v>
@@ -690,34 +792,34 @@
         <v>33</v>
       </c>
       <c r="I9" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J9" s="0">
         <v>6</v>
       </c>
       <c r="K9" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L9" s="0">
-        <v>16.805806208933358</v>
+        <v>16.693977074534551</v>
       </c>
       <c r="M9" s="0">
-        <v>16.824706797863996</v>
+        <v>16.717343900122078</v>
       </c>
       <c r="N9" s="0">
-        <v>99.673333333333332</v>
+        <v>99.921999999999997</v>
       </c>
       <c r="O9" s="0">
-        <v>99.59999999999998</v>
+        <v>99.859999999999985</v>
       </c>
       <c r="P9" s="0">
-        <v>41.666666666666664</v>
+        <v>27.199999999999999</v>
       </c>
       <c r="Q9" s="0">
-        <v>35.666666666666664</v>
+        <v>21.199999999999999</v>
       </c>
       <c r="R9" s="0">
-        <v>0.54466666666666919</v>
+        <v>0.74849999999999861</v>
       </c>
     </row>
     <row r="10">
@@ -725,16 +827,16 @@
         <v>9</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="C10" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D10" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>24</v>
+        <v>77</v>
       </c>
       <c r="F10" s="0" t="s">
         <v>27</v>
@@ -743,7 +845,7 @@
         <v>30</v>
       </c>
       <c r="H10" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I10" s="0" t="s">
         <v>35</v>
@@ -752,28 +854,28 @@
         <v>6</v>
       </c>
       <c r="K10" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L10" s="0">
-        <v>16.718757404520666</v>
+        <v>16.682416946041396</v>
       </c>
       <c r="M10" s="0">
-        <v>16.782255976279725</v>
+        <v>16.717638943220599</v>
       </c>
       <c r="N10" s="0">
-        <v>99.826666666666668</v>
+        <v>99.962000000000018</v>
       </c>
       <c r="O10" s="0">
-        <v>99.511111111111106</v>
+        <v>99.853333333333325</v>
       </c>
       <c r="P10" s="0">
-        <v>22.666666666666668</v>
+        <v>29.899999999999999</v>
       </c>
       <c r="Q10" s="0">
-        <v>16.666666666666668</v>
+        <v>23.899999999999999</v>
       </c>
       <c r="R10" s="0">
-        <v>0.50966666666666782</v>
+        <v>0.98610000000000042</v>
       </c>
     </row>
     <row r="11">
@@ -781,16 +883,16 @@
         <v>10</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C11" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D11" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E11" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F11" s="0" t="s">
         <v>28</v>
@@ -808,28 +910,28 @@
         <v>6</v>
       </c>
       <c r="K11" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L11" s="0">
-        <v>16.743861626262085</v>
+        <v>16.69425974659783</v>
       </c>
       <c r="M11" s="0">
-        <v>16.834489777975492</v>
+        <v>16.717304690619848</v>
       </c>
       <c r="N11" s="0">
-        <v>99.819999999999993</v>
+        <v>99.921999999999997</v>
       </c>
       <c r="O11" s="0">
-        <v>99.511111111111106</v>
+        <v>99.840000000000003</v>
       </c>
       <c r="P11" s="0">
-        <v>31</v>
+        <v>44.799999999999997</v>
       </c>
       <c r="Q11" s="0">
-        <v>25</v>
+        <v>40.299999999999997</v>
       </c>
       <c r="R11" s="0">
-        <v>0.25366666666666521</v>
+        <v>0.64609999999999912</v>
       </c>
     </row>
     <row r="12">
@@ -837,19 +939,19 @@
         <v>11</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>11</v>
+        <v>48</v>
       </c>
       <c r="C12" s="0" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D12" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E12" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F12" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G12" s="0" t="s">
         <v>30</v>
@@ -858,34 +960,34 @@
         <v>33</v>
       </c>
       <c r="I12" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J12" s="0">
         <v>6</v>
       </c>
       <c r="K12" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L12" s="0">
-        <v>16.753969495594962</v>
+        <v>16.711515657472681</v>
       </c>
       <c r="M12" s="0">
-        <v>16.836938974768796</v>
+        <v>16.741641274338957</v>
       </c>
       <c r="N12" s="0">
-        <v>99.766666666666666</v>
+        <v>99.889999999999986</v>
       </c>
       <c r="O12" s="0">
-        <v>99.511111111111106</v>
+        <v>99.799999999999983</v>
       </c>
       <c r="P12" s="0">
-        <v>15.333333333333334</v>
+        <v>33.399999999999999</v>
       </c>
       <c r="Q12" s="0">
-        <v>9.3333333333333339</v>
+        <v>27.899999999999999</v>
       </c>
       <c r="R12" s="0">
-        <v>0.33900000000000102</v>
+        <v>0.47930000000000062</v>
       </c>
     </row>
     <row r="13">
@@ -893,7 +995,7 @@
         <v>12</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>17</v>
+        <v>59</v>
       </c>
       <c r="C13" s="0" t="s">
         <v>20</v>
@@ -905,7 +1007,7 @@
         <v>24</v>
       </c>
       <c r="F13" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G13" s="0" t="s">
         <v>30</v>
@@ -914,34 +1016,34 @@
         <v>32</v>
       </c>
       <c r="I13" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J13" s="0">
         <v>6</v>
       </c>
       <c r="K13" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L13" s="0">
-        <v>16.725309533267431</v>
+        <v>16.721192564087435</v>
       </c>
       <c r="M13" s="0">
-        <v>16.795290728197219</v>
+        <v>16.759838056113264</v>
       </c>
       <c r="N13" s="0">
-        <v>99.806666666666672</v>
+        <v>99.816000000000003</v>
       </c>
       <c r="O13" s="0">
-        <v>99.466666666666654</v>
+        <v>99.690000000000012</v>
       </c>
       <c r="P13" s="0">
-        <v>45.666666666666664</v>
+        <v>22.399999999999999</v>
       </c>
       <c r="Q13" s="0">
-        <v>39.666666666666664</v>
+        <v>16.399999999999999</v>
       </c>
       <c r="R13" s="0">
-        <v>0.38166666666666771</v>
+        <v>0.56659999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -949,7 +1051,7 @@
         <v>13</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>8</v>
+        <v>56</v>
       </c>
       <c r="C14" s="0" t="s">
         <v>20</v>
@@ -958,16 +1060,16 @@
         <v>22</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="F14" s="0" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G14" s="0" t="s">
         <v>30</v>
       </c>
       <c r="H14" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I14" s="0" t="s">
         <v>35</v>
@@ -976,28 +1078,28 @@
         <v>6</v>
       </c>
       <c r="K14" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L14" s="0">
-        <v>16.826075850511906</v>
+        <v>16.728235577608153</v>
       </c>
       <c r="M14" s="0">
-        <v>16.925864087692688</v>
+        <v>16.772979574570417</v>
       </c>
       <c r="N14" s="0">
-        <v>99.420000000000002</v>
+        <v>99.847999999999999</v>
       </c>
       <c r="O14" s="0">
-        <v>99.155555555555551</v>
+        <v>99.653333333333336</v>
       </c>
       <c r="P14" s="0">
-        <v>21.666666666666668</v>
+        <v>39.899999999999999</v>
       </c>
       <c r="Q14" s="0">
-        <v>15.666666666666666</v>
+        <v>34.5</v>
       </c>
       <c r="R14" s="0">
-        <v>0.53633333333333155</v>
+        <v>0.3903999999999993</v>
       </c>
     </row>
     <row r="15">
@@ -1005,25 +1107,25 @@
         <v>14</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="C15" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D15" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F15" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G15" s="0" t="s">
         <v>30</v>
       </c>
       <c r="H15" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I15" s="0" t="s">
         <v>35</v>
@@ -1032,28 +1134,28 @@
         <v>6</v>
       </c>
       <c r="K15" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L15" s="0">
-        <v>17.609276797336346</v>
+        <v>16.747963789709054</v>
       </c>
       <c r="M15" s="0">
-        <v>17.605489518704477</v>
+        <v>16.777475187201731</v>
       </c>
       <c r="N15" s="0">
-        <v>89.799999999999997</v>
+        <v>99.773999999999987</v>
       </c>
       <c r="O15" s="0">
-        <v>89.600000000000009</v>
+        <v>99.640000000000015</v>
       </c>
       <c r="P15" s="0">
-        <v>36.333333333333336</v>
+        <v>19.100000000000001</v>
       </c>
       <c r="Q15" s="0">
-        <v>32.333333333333336</v>
+        <v>13.1</v>
       </c>
       <c r="R15" s="0">
-        <v>0.30700000000000216</v>
+        <v>0.54569999999999996</v>
       </c>
     </row>
     <row r="16">
@@ -1061,7 +1163,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>15</v>
+        <v>58</v>
       </c>
       <c r="C16" s="0" t="s">
         <v>20</v>
@@ -1070,46 +1172,46 @@
         <v>22</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F16" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G16" s="0" t="s">
         <v>30</v>
       </c>
       <c r="H16" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I16" s="0" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="J16" s="0">
         <v>6</v>
       </c>
       <c r="K16" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L16" s="0">
-        <v>18.661633047302303</v>
+        <v>16.755356827786027</v>
       </c>
       <c r="M16" s="0">
-        <v>18.785557209858975</v>
+        <v>16.81012425935015</v>
       </c>
       <c r="N16" s="0">
-        <v>77.24666666666667</v>
+        <v>99.766000000000005</v>
       </c>
       <c r="O16" s="0">
-        <v>76.400000000000006</v>
+        <v>99.570000000000007</v>
       </c>
       <c r="P16" s="0">
-        <v>41.333333333333336</v>
+        <v>25.399999999999999</v>
       </c>
       <c r="Q16" s="0">
-        <v>35.333333333333336</v>
+        <v>19.399999999999999</v>
       </c>
       <c r="R16" s="0">
-        <v>0.5579999999999975</v>
+        <v>0.66449999999999965</v>
       </c>
     </row>
     <row r="17">
@@ -1117,25 +1219,25 @@
         <v>16</v>
       </c>
       <c r="B17" s="0" t="s">
-        <v>13</v>
+        <v>60</v>
       </c>
       <c r="C17" s="0" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="D17" s="0" t="s">
         <v>22</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>25</v>
+        <v>77</v>
       </c>
       <c r="F17" s="0" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G17" s="0" t="s">
         <v>30</v>
       </c>
       <c r="H17" s="0" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="I17" s="0" t="s">
         <v>35</v>
@@ -1144,28 +1246,1820 @@
         <v>6</v>
       </c>
       <c r="K17" s="0">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="L17" s="0">
-        <v>19.452440703772712</v>
+        <v>16.737654942641246</v>
       </c>
       <c r="M17" s="0">
-        <v>19.507529210429137</v>
+        <v>16.81516258524292</v>
       </c>
       <c r="N17" s="0">
-        <v>72.879999999999996</v>
+        <v>99.825999999999993</v>
       </c>
       <c r="O17" s="0">
-        <v>72.711111111111109</v>
+        <v>99.560000000000016</v>
       </c>
       <c r="P17" s="0">
+        <v>16</v>
+      </c>
+      <c r="Q17" s="0">
+        <v>10</v>
+      </c>
+      <c r="R17" s="0">
+        <v>0.52560000000000007</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="0">
+        <v>17</v>
+      </c>
+      <c r="B18" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="C18" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E18" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G18" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H18" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I18" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J18" s="0">
+        <v>6</v>
+      </c>
+      <c r="K18" s="0">
+        <v>10</v>
+      </c>
+      <c r="L18" s="0">
+        <v>16.730862933864611</v>
+      </c>
+      <c r="M18" s="0">
+        <v>16.789714040762956</v>
+      </c>
+      <c r="N18" s="0">
+        <v>99.778000000000006</v>
+      </c>
+      <c r="O18" s="0">
+        <v>99.560000000000002</v>
+      </c>
+      <c r="P18" s="0">
+        <v>20.699999999999999</v>
+      </c>
+      <c r="Q18" s="0">
+        <v>14.699999999999999</v>
+      </c>
+      <c r="R18" s="0">
+        <v>0.52900000000000014</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="0">
+        <v>18</v>
+      </c>
+      <c r="B19" s="0" t="s">
+        <v>9</v>
+      </c>
+      <c r="C19" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E19" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G19" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H19" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I19" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J19" s="0">
+        <v>6</v>
+      </c>
+      <c r="K19" s="0">
+        <v>10</v>
+      </c>
+      <c r="L19" s="0">
+        <v>16.748230882744586</v>
+      </c>
+      <c r="M19" s="0">
+        <v>16.822061410558003</v>
+      </c>
+      <c r="N19" s="0">
+        <v>99.801999999999992</v>
+      </c>
+      <c r="O19" s="0">
+        <v>99.546666666666695</v>
+      </c>
+      <c r="P19" s="0">
+        <v>34.100000000000001</v>
+      </c>
+      <c r="Q19" s="0">
+        <v>27.899999999999999</v>
+      </c>
+      <c r="R19" s="0">
+        <v>0.31240000000000023</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="0">
+        <v>19</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="C20" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E20" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G20" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H20" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I20" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J20" s="0">
+        <v>6</v>
+      </c>
+      <c r="K20" s="0">
+        <v>10</v>
+      </c>
+      <c r="L20" s="0">
+        <v>16.745909135523014</v>
+      </c>
+      <c r="M20" s="0">
+        <v>16.810772970358137</v>
+      </c>
+      <c r="N20" s="0">
+        <v>99.787999999999983</v>
+      </c>
+      <c r="O20" s="0">
+        <v>99.540000000000006</v>
+      </c>
+      <c r="P20" s="0">
+        <v>34.100000000000001</v>
+      </c>
+      <c r="Q20" s="0">
+        <v>28.100000000000001</v>
+      </c>
+      <c r="R20" s="0">
+        <v>0.30530000000000185</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="0">
+        <v>20</v>
+      </c>
+      <c r="B21" s="0" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E21" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F21" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H21" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I21" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J21" s="0">
+        <v>6</v>
+      </c>
+      <c r="K21" s="0">
+        <v>10</v>
+      </c>
+      <c r="L21" s="0">
+        <v>16.756761672883094</v>
+      </c>
+      <c r="M21" s="0">
+        <v>16.815672287084027</v>
+      </c>
+      <c r="N21" s="0">
+        <v>99.739999999999995</v>
+      </c>
+      <c r="O21" s="0">
+        <v>99.540000000000006</v>
+      </c>
+      <c r="P21" s="0">
+        <v>20.699999999999999</v>
+      </c>
+      <c r="Q21" s="0">
+        <v>14.699999999999999</v>
+      </c>
+      <c r="R21" s="0">
+        <v>0.58179999999999976</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="0">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E22" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G22" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H22" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I22" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J22" s="0">
+        <v>6</v>
+      </c>
+      <c r="K22" s="0">
+        <v>10</v>
+      </c>
+      <c r="L22" s="0">
+        <v>16.749452429182043</v>
+      </c>
+      <c r="M22" s="0">
+        <v>16.826380683686718</v>
+      </c>
+      <c r="N22" s="0">
+        <v>99.796000000000007</v>
+      </c>
+      <c r="O22" s="0">
+        <v>99.533333333333346</v>
+      </c>
+      <c r="P22" s="0">
+        <v>30</v>
+      </c>
+      <c r="Q22" s="0">
+        <v>24</v>
+      </c>
+      <c r="R22" s="0">
+        <v>0.77529999999999999</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="0">
+        <v>22</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>63</v>
       </c>
-      <c r="Q17" s="0">
-        <v>61</v>
-      </c>
-      <c r="R17" s="0">
-        <v>0.84833333333333394</v>
+      <c r="C23" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E23" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F23" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H23" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I23" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J23" s="0">
+        <v>6</v>
+      </c>
+      <c r="K23" s="0">
+        <v>10</v>
+      </c>
+      <c r="L23" s="0">
+        <v>16.790744886371769</v>
+      </c>
+      <c r="M23" s="0">
+        <v>16.84542911926345</v>
+      </c>
+      <c r="N23" s="0">
+        <v>99.675999999999988</v>
+      </c>
+      <c r="O23" s="0">
+        <v>99.480000000000004</v>
+      </c>
+      <c r="P23" s="0">
+        <v>35.600000000000001</v>
+      </c>
+      <c r="Q23" s="0">
+        <v>29.600000000000001</v>
+      </c>
+      <c r="R23" s="0">
+        <v>0.52700000000000102</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="0">
+        <v>23</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>66</v>
+      </c>
+      <c r="C24" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E24" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F24" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G24" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H24" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I24" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J24" s="0">
+        <v>6</v>
+      </c>
+      <c r="K24" s="0">
+        <v>10</v>
+      </c>
+      <c r="L24" s="0">
+        <v>16.726030901338437</v>
+      </c>
+      <c r="M24" s="0">
+        <v>16.800847322701738</v>
+      </c>
+      <c r="N24" s="0">
+        <v>99.774000000000001</v>
+      </c>
+      <c r="O24" s="0">
+        <v>99.460000000000008</v>
+      </c>
+      <c r="P24" s="0">
+        <v>22.899999999999999</v>
+      </c>
+      <c r="Q24" s="0">
+        <v>16.899999999999999</v>
+      </c>
+      <c r="R24" s="0">
+        <v>0.73959999999999948</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="0">
+        <v>24</v>
+      </c>
+      <c r="B25" s="0" t="s">
+        <v>62</v>
+      </c>
+      <c r="C25" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E25" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F25" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G25" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H25" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I25" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J25" s="0">
+        <v>6</v>
+      </c>
+      <c r="K25" s="0">
+        <v>10</v>
+      </c>
+      <c r="L25" s="0">
+        <v>16.752532555655851</v>
+      </c>
+      <c r="M25" s="0">
+        <v>16.847434381309977</v>
+      </c>
+      <c r="N25" s="0">
+        <v>99.772000000000006</v>
+      </c>
+      <c r="O25" s="0">
+        <v>99.439999999999998</v>
+      </c>
+      <c r="P25" s="0">
+        <v>35</v>
+      </c>
+      <c r="Q25" s="0">
+        <v>29</v>
+      </c>
+      <c r="R25" s="0">
+        <v>1.1536</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="0">
+        <v>25</v>
+      </c>
+      <c r="B26" s="0" t="s">
+        <v>64</v>
+      </c>
+      <c r="C26" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E26" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G26" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H26" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I26" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J26" s="0">
+        <v>6</v>
+      </c>
+      <c r="K26" s="0">
+        <v>10</v>
+      </c>
+      <c r="L26" s="0">
+        <v>17.252360739293096</v>
+      </c>
+      <c r="M26" s="0">
+        <v>17.264278983374886</v>
+      </c>
+      <c r="N26" s="0">
+        <v>98.301999999999992</v>
+      </c>
+      <c r="O26" s="0">
+        <v>98.239999999999995</v>
+      </c>
+      <c r="P26" s="0">
+        <v>30.800000000000001</v>
+      </c>
+      <c r="Q26" s="0">
+        <v>24.800000000000001</v>
+      </c>
+      <c r="R26" s="0">
+        <v>0.31549999999999939</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="0">
+        <v>26</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>54</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D27" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E27" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F27" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H27" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I27" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J27" s="0">
+        <v>6</v>
+      </c>
+      <c r="K27" s="0">
+        <v>10</v>
+      </c>
+      <c r="L27" s="0">
+        <v>17.258168726588796</v>
+      </c>
+      <c r="M27" s="0">
+        <v>17.274336067581018</v>
+      </c>
+      <c r="N27" s="0">
+        <v>98.224000000000004</v>
+      </c>
+      <c r="O27" s="0">
+        <v>98.169999999999987</v>
+      </c>
+      <c r="P27" s="0">
+        <v>38.799999999999997</v>
+      </c>
+      <c r="Q27" s="0">
+        <v>35.700000000000003</v>
+      </c>
+      <c r="R27" s="0">
+        <v>0.3847999999999992</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="0">
+        <v>27</v>
+      </c>
+      <c r="B28" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D28" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E28" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F28" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G28" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H28" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I28" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J28" s="0">
+        <v>6</v>
+      </c>
+      <c r="K28" s="0">
+        <v>10</v>
+      </c>
+      <c r="L28" s="0">
+        <v>16.952137822030128</v>
+      </c>
+      <c r="M28" s="0">
+        <v>16.95209144373759</v>
+      </c>
+      <c r="N28" s="0">
+        <v>96.618000000000009</v>
+      </c>
+      <c r="O28" s="0">
+        <v>96.693333333333342</v>
+      </c>
+      <c r="P28" s="0">
+        <v>21</v>
+      </c>
+      <c r="Q28" s="0">
+        <v>17.300000000000001</v>
+      </c>
+      <c r="R28" s="0">
+        <v>0.69100000000000039</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="0">
+        <v>28</v>
+      </c>
+      <c r="B29" s="0" t="s">
+        <v>53</v>
+      </c>
+      <c r="C29" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D29" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G29" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H29" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I29" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J29" s="0">
+        <v>6</v>
+      </c>
+      <c r="K29" s="0">
+        <v>10</v>
+      </c>
+      <c r="L29" s="0">
+        <v>16.958284416516669</v>
+      </c>
+      <c r="M29" s="0">
+        <v>16.963707953692207</v>
+      </c>
+      <c r="N29" s="0">
+        <v>96.612000000000009</v>
+      </c>
+      <c r="O29" s="0">
+        <v>96.679999999999978</v>
+      </c>
+      <c r="P29" s="0">
+        <v>16.800000000000001</v>
+      </c>
+      <c r="Q29" s="0">
+        <v>12.800000000000001</v>
+      </c>
+      <c r="R29" s="0">
+        <v>0.41720000000000185</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="0">
+        <v>29</v>
+      </c>
+      <c r="B30" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D30" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E30" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F30" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G30" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H30" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I30" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J30" s="0">
+        <v>6</v>
+      </c>
+      <c r="K30" s="0">
+        <v>10</v>
+      </c>
+      <c r="L30" s="0">
+        <v>17.648985669099361</v>
+      </c>
+      <c r="M30" s="0">
+        <v>17.688398615652549</v>
+      </c>
+      <c r="N30" s="0">
+        <v>96.646000000000001</v>
+      </c>
+      <c r="O30" s="0">
+        <v>96.52000000000001</v>
+      </c>
+      <c r="P30" s="0">
+        <v>31.899999999999999</v>
+      </c>
+      <c r="Q30" s="0">
+        <v>28.699999999999999</v>
+      </c>
+      <c r="R30" s="0">
+        <v>0.32179999999999931</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="0">
+        <v>30</v>
+      </c>
+      <c r="B31" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="C31" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D31" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E31" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F31" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G31" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H31" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I31" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J31" s="0">
+        <v>6</v>
+      </c>
+      <c r="K31" s="0">
+        <v>10</v>
+      </c>
+      <c r="L31" s="0">
+        <v>17.807103113092676</v>
+      </c>
+      <c r="M31" s="0">
+        <v>17.86704513316851</v>
+      </c>
+      <c r="N31" s="0">
+        <v>96.586000000000013</v>
+      </c>
+      <c r="O31" s="0">
+        <v>96.413333333333327</v>
+      </c>
+      <c r="P31" s="0">
+        <v>30.199999999999999</v>
+      </c>
+      <c r="Q31" s="0">
+        <v>24.699999999999999</v>
+      </c>
+      <c r="R31" s="0">
+        <v>0.81780000000000042</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="0">
+        <v>31</v>
+      </c>
+      <c r="B32" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E32" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F32" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G32" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H32" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="I32" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J32" s="0">
+        <v>6</v>
+      </c>
+      <c r="K32" s="0">
+        <v>10</v>
+      </c>
+      <c r="L32" s="0">
+        <v>17.753208181414898</v>
+      </c>
+      <c r="M32" s="0">
+        <v>17.786112397050893</v>
+      </c>
+      <c r="N32" s="0">
+        <v>96.402000000000001</v>
+      </c>
+      <c r="O32" s="0">
+        <v>96.293333333333337</v>
+      </c>
+      <c r="P32" s="0">
+        <v>32.299999999999997</v>
+      </c>
+      <c r="Q32" s="0">
+        <v>26.100000000000001</v>
+      </c>
+      <c r="R32" s="0">
+        <v>0.46029999999999804</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="0">
+        <v>32</v>
+      </c>
+      <c r="B33" s="0" t="s">
+        <v>75</v>
+      </c>
+      <c r="C33" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E33" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F33" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H33" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I33" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J33" s="0">
+        <v>6</v>
+      </c>
+      <c r="K33" s="0">
+        <v>10</v>
+      </c>
+      <c r="L33" s="0">
+        <v>17.287579110867622</v>
+      </c>
+      <c r="M33" s="0">
+        <v>17.333387357350901</v>
+      </c>
+      <c r="N33" s="0">
+        <v>96.295999999999992</v>
+      </c>
+      <c r="O33" s="0">
+        <v>96.210000000000008</v>
+      </c>
+      <c r="P33" s="0">
+        <v>20.300000000000001</v>
+      </c>
+      <c r="Q33" s="0">
+        <v>14.300000000000001</v>
+      </c>
+      <c r="R33" s="0">
+        <v>0.55199999999999905</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="0">
+        <v>33</v>
+      </c>
+      <c r="B34" s="0" t="s">
+        <v>68</v>
+      </c>
+      <c r="C34" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E34" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F34" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H34" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I34" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J34" s="0">
+        <v>6</v>
+      </c>
+      <c r="K34" s="0">
+        <v>10</v>
+      </c>
+      <c r="L34" s="0">
+        <v>17.291153973734367</v>
+      </c>
+      <c r="M34" s="0">
+        <v>17.361740396072385</v>
+      </c>
+      <c r="N34" s="0">
+        <v>94.436000000000007</v>
+      </c>
+      <c r="O34" s="0">
+        <v>94.159999999999997</v>
+      </c>
+      <c r="P34" s="0">
+        <v>46.700000000000003</v>
+      </c>
+      <c r="Q34" s="0">
+        <v>40.700000000000003</v>
+      </c>
+      <c r="R34" s="0">
+        <v>0.42210000000000036</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="0">
+        <v>34</v>
+      </c>
+      <c r="B35" s="0" t="s">
+        <v>16</v>
+      </c>
+      <c r="C35" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D35" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E35" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F35" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G35" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H35" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I35" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J35" s="0">
+        <v>6</v>
+      </c>
+      <c r="K35" s="0">
+        <v>10</v>
+      </c>
+      <c r="L35" s="0">
+        <v>17.232339879876058</v>
+      </c>
+      <c r="M35" s="0">
+        <v>17.242973663972965</v>
+      </c>
+      <c r="N35" s="0">
+        <v>93.256</v>
+      </c>
+      <c r="O35" s="0">
+        <v>93.186666666666682</v>
+      </c>
+      <c r="P35" s="0">
+        <v>22</v>
+      </c>
+      <c r="Q35" s="0">
+        <v>19.199999999999999</v>
+      </c>
+      <c r="R35" s="0">
+        <v>0.57430000000000026</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="0">
+        <v>35</v>
+      </c>
+      <c r="B36" s="0" t="s">
+        <v>4</v>
+      </c>
+      <c r="C36" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E36" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H36" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I36" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J36" s="0">
+        <v>6</v>
+      </c>
+      <c r="K36" s="0">
+        <v>10</v>
+      </c>
+      <c r="L36" s="0">
+        <v>17.518477139212038</v>
+      </c>
+      <c r="M36" s="0">
+        <v>17.535736070274947</v>
+      </c>
+      <c r="N36" s="0">
+        <v>92.994</v>
+      </c>
+      <c r="O36" s="0">
+        <v>92.733333333333334</v>
+      </c>
+      <c r="P36" s="0">
+        <v>50.799999999999997</v>
+      </c>
+      <c r="Q36" s="0">
+        <v>45.299999999999997</v>
+      </c>
+      <c r="R36" s="0">
+        <v>0.44860000000000017</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="0">
+        <v>36</v>
+      </c>
+      <c r="B37" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="C37" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E37" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F37" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G37" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H37" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I37" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J37" s="0">
+        <v>6</v>
+      </c>
+      <c r="K37" s="0">
+        <v>10</v>
+      </c>
+      <c r="L37" s="0">
+        <v>17.277330937327065</v>
+      </c>
+      <c r="M37" s="0">
+        <v>17.364391348531324</v>
+      </c>
+      <c r="N37" s="0">
+        <v>93.099999999999994</v>
+      </c>
+      <c r="O37" s="0">
+        <v>92.666666666666686</v>
+      </c>
+      <c r="P37" s="0">
+        <v>24.199999999999999</v>
+      </c>
+      <c r="Q37" s="0">
+        <v>18.199999999999999</v>
+      </c>
+      <c r="R37" s="0">
+        <v>0.78489999999999893</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="0">
+        <v>37</v>
+      </c>
+      <c r="B38" s="0" t="s">
+        <v>70</v>
+      </c>
+      <c r="C38" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D38" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E38" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F38" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G38" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H38" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I38" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J38" s="0">
+        <v>6</v>
+      </c>
+      <c r="K38" s="0">
+        <v>10</v>
+      </c>
+      <c r="L38" s="0">
+        <v>17.511101276620959</v>
+      </c>
+      <c r="M38" s="0">
+        <v>17.529189434226147</v>
+      </c>
+      <c r="N38" s="0">
+        <v>92.256</v>
+      </c>
+      <c r="O38" s="0">
+        <v>92.039999999999992</v>
+      </c>
+      <c r="P38" s="0">
+        <v>42.5</v>
+      </c>
+      <c r="Q38" s="0">
+        <v>37</v>
+      </c>
+      <c r="R38" s="0">
+        <v>0.38249999999999995</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="0">
+        <v>38</v>
+      </c>
+      <c r="B39" s="0" t="s">
+        <v>69</v>
+      </c>
+      <c r="C39" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E39" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F39" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G39" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H39" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I39" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J39" s="0">
+        <v>6</v>
+      </c>
+      <c r="K39" s="0">
+        <v>10</v>
+      </c>
+      <c r="L39" s="0">
+        <v>17.82513527309629</v>
+      </c>
+      <c r="M39" s="0">
+        <v>17.874840088747302</v>
+      </c>
+      <c r="N39" s="0">
+        <v>90.161999999999992</v>
+      </c>
+      <c r="O39" s="0">
+        <v>90.22999999999999</v>
+      </c>
+      <c r="P39" s="0">
+        <v>41.5</v>
+      </c>
+      <c r="Q39" s="0">
+        <v>35.399999999999999</v>
+      </c>
+      <c r="R39" s="0">
+        <v>0.39649999999999963</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="0">
+        <v>39</v>
+      </c>
+      <c r="B40" s="0" t="s">
+        <v>67</v>
+      </c>
+      <c r="C40" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D40" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E40" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F40" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G40" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H40" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I40" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J40" s="0">
+        <v>6</v>
+      </c>
+      <c r="K40" s="0">
+        <v>10</v>
+      </c>
+      <c r="L40" s="0">
+        <v>17.56288609484886</v>
+      </c>
+      <c r="M40" s="0">
+        <v>17.620305074665826</v>
+      </c>
+      <c r="N40" s="0">
+        <v>90.35799999999999</v>
+      </c>
+      <c r="O40" s="0">
+        <v>90.213333333333324</v>
+      </c>
+      <c r="P40" s="0">
+        <v>49.100000000000001</v>
+      </c>
+      <c r="Q40" s="0">
+        <v>43.100000000000001</v>
+      </c>
+      <c r="R40" s="0">
+        <v>0.47759999999999964</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="0">
+        <v>40</v>
+      </c>
+      <c r="B41" s="0" t="s">
+        <v>73</v>
+      </c>
+      <c r="C41" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D41" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E41" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F41" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G41" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H41" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I41" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J41" s="0">
+        <v>6</v>
+      </c>
+      <c r="K41" s="0">
+        <v>10</v>
+      </c>
+      <c r="L41" s="0">
+        <v>17.78555895558582</v>
+      </c>
+      <c r="M41" s="0">
+        <v>17.808997557107794</v>
+      </c>
+      <c r="N41" s="0">
+        <v>89.921999999999997</v>
+      </c>
+      <c r="O41" s="0">
+        <v>89.810000000000002</v>
+      </c>
+      <c r="P41" s="0">
+        <v>45.299999999999997</v>
+      </c>
+      <c r="Q41" s="0">
+        <v>40.5</v>
+      </c>
+      <c r="R41" s="0">
+        <v>0.42350000000000032</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="0">
+        <v>41</v>
+      </c>
+      <c r="B42" s="0" t="s">
+        <v>71</v>
+      </c>
+      <c r="C42" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D42" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E42" s="0" t="s">
+        <v>77</v>
+      </c>
+      <c r="F42" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G42" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H42" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I42" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J42" s="0">
+        <v>6</v>
+      </c>
+      <c r="K42" s="0">
+        <v>10</v>
+      </c>
+      <c r="L42" s="0">
+        <v>18.043521029836828</v>
+      </c>
+      <c r="M42" s="0">
+        <v>18.041582241703697</v>
+      </c>
+      <c r="N42" s="0">
+        <v>87.746000000000009</v>
+      </c>
+      <c r="O42" s="0">
+        <v>87.74666666666667</v>
+      </c>
+      <c r="P42" s="0">
+        <v>51.899999999999999</v>
+      </c>
+      <c r="Q42" s="0">
+        <v>48.700000000000003</v>
+      </c>
+      <c r="R42" s="0">
+        <v>0.51550000000000007</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="0">
+        <v>42</v>
+      </c>
+      <c r="B43" s="0" t="s">
+        <v>72</v>
+      </c>
+      <c r="C43" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D43" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E43" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F43" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G43" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H43" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I43" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J43" s="0">
+        <v>6</v>
+      </c>
+      <c r="K43" s="0">
+        <v>10</v>
+      </c>
+      <c r="L43" s="0">
+        <v>17.786171111832538</v>
+      </c>
+      <c r="M43" s="0">
+        <v>17.790283604736643</v>
+      </c>
+      <c r="N43" s="0">
+        <v>86.632000000000019</v>
+      </c>
+      <c r="O43" s="0">
+        <v>86.679999999999993</v>
+      </c>
+      <c r="P43" s="0">
+        <v>61.700000000000003</v>
+      </c>
+      <c r="Q43" s="0">
+        <v>59.299999999999997</v>
+      </c>
+      <c r="R43" s="0">
+        <v>1.670699999999999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="0">
+        <v>43</v>
+      </c>
+      <c r="B44" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="C44" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D44" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E44" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F44" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="G44" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H44" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I44" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J44" s="0">
+        <v>6</v>
+      </c>
+      <c r="K44" s="0">
+        <v>10</v>
+      </c>
+      <c r="L44" s="0">
+        <v>18.383148501406918</v>
+      </c>
+      <c r="M44" s="0">
+        <v>18.438343884167658</v>
+      </c>
+      <c r="N44" s="0">
+        <v>86.47199999999998</v>
+      </c>
+      <c r="O44" s="0">
+        <v>86.093333333333334</v>
+      </c>
+      <c r="P44" s="0">
+        <v>26.699999999999999</v>
+      </c>
+      <c r="Q44" s="0">
+        <v>21</v>
+      </c>
+      <c r="R44" s="0">
+        <v>0.73970000000000058</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="0">
+        <v>44</v>
+      </c>
+      <c r="B45" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="C45" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D45" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E45" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F45" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G45" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H45" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I45" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J45" s="0">
+        <v>6</v>
+      </c>
+      <c r="K45" s="0">
+        <v>10</v>
+      </c>
+      <c r="L45" s="0">
+        <v>18.35873757952735</v>
+      </c>
+      <c r="M45" s="0">
+        <v>18.430236199447311</v>
+      </c>
+      <c r="N45" s="0">
+        <v>83.126000000000005</v>
+      </c>
+      <c r="O45" s="0">
+        <v>82.493333333333339</v>
+      </c>
+      <c r="P45" s="0">
+        <v>54.700000000000003</v>
+      </c>
+      <c r="Q45" s="0">
+        <v>49.200000000000003</v>
+      </c>
+      <c r="R45" s="0">
+        <v>0.77969999999999995</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="0">
+        <v>45</v>
+      </c>
+      <c r="B46" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D46" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E46" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F46" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G46" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H46" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I46" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J46" s="0">
+        <v>6</v>
+      </c>
+      <c r="K46" s="0">
+        <v>10</v>
+      </c>
+      <c r="L46" s="0">
+        <v>18.68559709831478</v>
+      </c>
+      <c r="M46" s="0">
+        <v>18.767509300078377</v>
+      </c>
+      <c r="N46" s="0">
+        <v>79.864000000000004</v>
+      </c>
+      <c r="O46" s="0">
+        <v>79.120000000000005</v>
+      </c>
+      <c r="P46" s="0">
+        <v>48.399999999999999</v>
+      </c>
+      <c r="Q46" s="0">
+        <v>42.399999999999999</v>
+      </c>
+      <c r="R46" s="0">
+        <v>0.68349999999999977</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="0">
+        <v>46</v>
+      </c>
+      <c r="B47" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C47" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D47" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E47" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="F47" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G47" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H47" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I47" s="0" t="s">
+        <v>35</v>
+      </c>
+      <c r="J47" s="0">
+        <v>6</v>
+      </c>
+      <c r="K47" s="0">
+        <v>10</v>
+      </c>
+      <c r="L47" s="0">
+        <v>18.682746015205971</v>
+      </c>
+      <c r="M47" s="0">
+        <v>18.755105573105361</v>
+      </c>
+      <c r="N47" s="0">
+        <v>77.332000000000022</v>
+      </c>
+      <c r="O47" s="0">
+        <v>76.86666666666666</v>
+      </c>
+      <c r="P47" s="0">
+        <v>42.100000000000001</v>
+      </c>
+      <c r="Q47" s="0">
+        <v>35.899999999999999</v>
+      </c>
+      <c r="R47" s="0">
+        <v>0.36310000000000076</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="0">
+        <v>47</v>
+      </c>
+      <c r="B48" s="0" t="s">
+        <v>74</v>
+      </c>
+      <c r="C48" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="D48" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E48" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F48" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G48" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H48" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I48" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J48" s="0">
+        <v>6</v>
+      </c>
+      <c r="K48" s="0">
+        <v>10</v>
+      </c>
+      <c r="L48" s="0">
+        <v>19.462737810139974</v>
+      </c>
+      <c r="M48" s="0">
+        <v>19.424952798146567</v>
+      </c>
+      <c r="N48" s="0">
+        <v>72.984000000000009</v>
+      </c>
+      <c r="O48" s="0">
+        <v>73.450000000000003</v>
+      </c>
+      <c r="P48" s="0">
+        <v>43.600000000000001</v>
+      </c>
+      <c r="Q48" s="0">
+        <v>37.5</v>
+      </c>
+      <c r="R48" s="0">
+        <v>0.61530000000000007</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="0">
+        <v>48</v>
+      </c>
+      <c r="B49" s="0" t="s">
+        <v>76</v>
+      </c>
+      <c r="C49" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="D49" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="E49" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="F49" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="G49" s="0" t="s">
+        <v>30</v>
+      </c>
+      <c r="H49" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="I49" s="0" t="s">
+        <v>78</v>
+      </c>
+      <c r="J49" s="0">
+        <v>6</v>
+      </c>
+      <c r="K49" s="0">
+        <v>10</v>
+      </c>
+      <c r="L49" s="0">
+        <v>20.625805523291014</v>
+      </c>
+      <c r="M49" s="0">
+        <v>20.672639150327065</v>
+      </c>
+      <c r="N49" s="0">
+        <v>69.189999999999984</v>
+      </c>
+      <c r="O49" s="0">
+        <v>69.300000000000011</v>
+      </c>
+      <c r="P49" s="0">
+        <v>42.100000000000001</v>
+      </c>
+      <c r="Q49" s="0">
+        <v>37.299999999999997</v>
+      </c>
+      <c r="R49" s="0">
+        <v>0.60579999999999967</v>
       </c>
     </row>
   </sheetData>

</xml_diff>